<commit_message>
fix: align Day25 completion and containment semantics
</commit_message>
<xml_diff>
--- a/deliverables/NguyenQuangHuy_Day25_model.xlsx
+++ b/deliverables/NguyenQuangHuy_Day25_model.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="0_README" sheetId="1" r:id="R21774baa25c54acf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1_Cost_Job" sheetId="2" r:id="R98a6d7f0d06441f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_Pricing" sheetId="3" r:id="R9fab25e88f1e4973"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_Value_Metric" sheetId="4" r:id="R201add8f1ec14e73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_Channel_Fit" sheetId="5" r:id="Rb60b9855dcf74bdd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_90Day_Plan" sheetId="6" r:id="Rfc0756833b854bc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6_Benchmarks" sheetId="7" r:id="R5e9d05239c69407e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="0_README" sheetId="1" r:id="R2f6804631e444d6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1_Cost_Job" sheetId="2" r:id="Rc2c96c01c88b4ff6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_Pricing" sheetId="3" r:id="R4f0fbbf238ce41e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_Value_Metric" sheetId="4" r:id="R072bf18d4d46451f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_Channel_Fit" sheetId="5" r:id="Rf878533bb2fb423e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_90Day_Plan" sheetId="6" r:id="Rd2f8519d599e489a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6_Benchmarks" sheetId="7" r:id="R875a1343d73c4eba"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,8 +16,8 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={F0DCF4DE-B7EE-1AD0-7C01-426A9C293E1E}</x:author>
-    <x:author>tc={3981B259-D4F8-F94D-A193-8AC8AD06418D}</x:author>
+    <x:author>tc={12804478-9915-33E9-BDEA-08B74E3B929F}</x:author>
+    <x:author>tc={52C99004-C050-8257-19BE-6EDA81ABA477}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="C26" authorId="0">
@@ -47,7 +47,7 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={DA39F2BA-FA9E-1663-750E-0E3FD6472E16}</x:author>
+    <x:author>tc={C05352F1-6581-C37C-4B99-163BCD33299C}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="C16" authorId="0">
@@ -56,7 +56,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Formula: solve direct_cost / (price x attempts x containment) &lt;= 1 - GM_target. QA cost per completion is included in the denominator adjustment.</x:t>
+    Formula: solve for the commercial package-completion rate p in direct_cost / (price x attempts x p, with QA cost per completed package) &lt;= 1 - GM_target. This is not an autonomous-containment threshold; local autonomous containment is 20%.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -609,7 +609,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Nguyen Quang Huy" id="{B543B0F2-B004-4167-B60F-8CCEE8E2DDDC}"/>
+  <xltc:person displayName="Nguyen Quang Huy" id="{651A636D-9806-49DD-9B61-45135D76737F}"/>
 </xltc:personList>
 </file>
 
@@ -806,10 +806,10 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="C26" dT="2026-08-27T02:44:20.601" personId="{B543B0F2-B004-4167-B60F-8CCEE8E2DDDC}" id="{F0DCF4DE-B7EE-1AD0-7C01-426A9C293E1E}">
+  <xltc:threadedComment ref="C26" dT="2026-08-27T03:00:18.985" personId="{651A636D-9806-49DD-9B61-45135D76737F}" id="{12804478-9915-33E9-BDEA-08B74E3B929F}">
     <xltc:text>Source: https://platform.openai.com/pricing?model=contentfilter-alpha-001 checked 2026-08-27. GPT-5.5 Standard short-context input price used in the base scenario.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="C44" dT="2026-08-27T02:44:20.602" personId="{B543B0F2-B004-4167-B60F-8CCEE8E2DDDC}" id="{3981B259-D4F8-F94D-A193-8AC8AD06418D}">
+  <xltc:threadedComment ref="C44" dT="2026-08-27T03:00:18.998" personId="{651A636D-9806-49DD-9B61-45135D76737F}" id="{52C99004-C050-8257-19BE-6EDA81ABA477}">
     <xltc:text>Source: https://supabase.com/pricing checked 2026-08-27. Pro plan is $25/month; additional app/compute/logging reserve is an explicit assumption.</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -817,8 +817,8 @@
 
 <file path=xl/threadedcomments/threadedcomment2.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="C16" dT="2026-08-27T02:44:20.602" personId="{B543B0F2-B004-4167-B60F-8CCEE8E2DDDC}" id="{DA39F2BA-FA9E-1663-750E-0E3FD6472E16}">
-    <xltc:text>Formula: solve direct_cost / (price x attempts x containment) &lt;= 1 - GM_target. QA cost per completion is included in the denominator adjustment.</xltc:text>
+  <xltc:threadedComment ref="C16" dT="2026-08-27T03:00:19" personId="{651A636D-9806-49DD-9B61-45135D76737F}" id="{C05352F1-6581-C37C-4B99-163BCD33299C}">
+    <xltc:text>Formula: solve for the commercial package-completion rate p in direct_cost / (price x attempts x p, with QA cost per completed package) &lt;= 1 - GM_target. This is not an autonomous-containment threshold; local autonomous containment is 20%.</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
 </file>
@@ -986,7 +986,7 @@
         <x:v>Critical caveat</x:v>
       </x:c>
       <x:c r="B12" s="72" t="str">
-        <x:v>Commercial completion / containment is an 80% LOCAL CONTROLLED EVAL PROXY from 4/5 grounded packages; it is not customer evidence. Autonomous completion in the same run is 20%.</x:v>
+        <x:v>Commercial package completion rate is 80% (4/5) in a LOCAL CONTROLLED EVAL; autonomous containment rate is 20% (1/5), human-review/escalation rate is 80% (4/5), and grounding failure rate is 20% (1/5). None is customer evidence.</x:v>
       </x:c>
       <x:c r="C12" s="72" t="str"/>
       <x:c r="D12" s="72" t="str"/>
@@ -1345,7 +1345,7 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="72" t="str">
-        <x:v>Completion / containment rate</x:v>
+        <x:v>Commercial package completion rate</x:v>
       </x:c>
       <x:c r="B7" s="72" t="str">
         <x:v>% of attempts</x:v>
@@ -1357,12 +1357,12 @@
         <x:v>LOCAL CONTROLLED EVAL</x:v>
       </x:c>
       <x:c r="E7" s="72" t="str">
-        <x:v>4/5 grounded, schema-valid commercial packages in evidence/containment-eval.md; not production customer completion. Autonomous completion in the same run is 1/5 (20%).</x:v>
+        <x:v>4/5 grounded, schema-valid commercial packages in evidence/containment-eval.md; not a customer rate. Separate local metrics: autonomous containment 1/5 (20%), human-review/escalation 4/5 (80%), grounding failure 1/5 (20%).</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="72" t="str">
-        <x:v>Completed jobs</x:v>
+        <x:v>Completed commercial jobs</x:v>
       </x:c>
       <x:c r="B8" s="72" t="str">
         <x:v>jobs / month</x:v>
@@ -1375,12 +1375,12 @@
         <x:v>FORMULA</x:v>
       </x:c>
       <x:c r="E8" s="72" t="str">
-        <x:v>Jobs attempted x completion rate. Denominator for Cost/Job.</x:v>
+        <x:v>Jobs attempted x commercial package-completion rate. Denominator for Cost/Job.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="72" t="str">
-        <x:v>Escalation rate</x:v>
+        <x:v>Modelled escalation rate</x:v>
       </x:c>
       <x:c r="B9" s="72" t="str">
         <x:v>% of completed</x:v>
@@ -1392,7 +1392,7 @@
         <x:v>ESTIMATE</x:v>
       </x:c>
       <x:c r="E9" s="72" t="str">
-        <x:v>Human review remains material; 4/5 local cases required review, but that sample is not a production rate.</x:v>
+        <x:v>Planning cost assumption; separate local controlled eval observed human-review/escalation in 4/5 cases (80%), not a production rate.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2365,7 +2365,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5eb86efb9c4b4fad"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b72ae4a503a410d"/>
 </x:worksheet>
 </file>
 
@@ -2613,7 +2613,7 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="72" t="str">
-        <x:v>Current / evaluated containment</x:v>
+        <x:v>Current commercial package completion rate</x:v>
       </x:c>
       <x:c r="B14" s="72" t="str">
         <x:v>%</x:v>
@@ -2626,7 +2626,7 @@
         <x:v>LOCAL CONTROLLED EVAL</x:v>
       </x:c>
       <x:c r="E14" s="72" t="str">
-        <x:v>Linked from Cost/Job: 4/5 grounded-package completion; separate autonomous completion is 20%; production containment remains unmeasured.</x:v>
+        <x:v>Linked from Cost/Job: 4/5 grounded-package completion (80%); autonomous containment is 1/5 (20%) and is not compared with the package-completion threshold.</x:v>
       </x:c>
       <x:c r="F14" s="68"/>
     </x:row>
@@ -2650,7 +2650,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="72" t="str">
-        <x:v>Required containment for GM target</x:v>
+        <x:v>Breakeven package-completion rate for GM target</x:v>
       </x:c>
       <x:c r="B16" s="72" t="str">
         <x:v>%</x:v>
@@ -2663,13 +2663,13 @@
         <x:v>FORMULA</x:v>
       </x:c>
       <x:c r="E16" s="72" t="str">
-        <x:v>Algebraic minimum at proposed usage price.</x:v>
+        <x:v>Algebraic minimum commercial package-completion rate at proposed usage price; not an autonomous-containment threshold.</x:v>
       </x:c>
       <x:c r="F16" s="68"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="72" t="str">
-        <x:v>Safety buffer</x:v>
+        <x:v>Package-completion buffer</x:v>
       </x:c>
       <x:c r="B17" s="72" t="str">
         <x:v>percentage points</x:v>
@@ -2682,13 +2682,13 @@
         <x:v>FORMULA</x:v>
       </x:c>
       <x:c r="E17" s="72" t="str">
-        <x:v>Controlled-eval commercial completion proxy less required containment.</x:v>
+        <x:v>Commercial package-completion rate less breakeven package-completion rate.</x:v>
       </x:c>
       <x:c r="F17" s="68"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="72" t="str">
-        <x:v>Containment error scenario</x:v>
+        <x:v>Package-completion error scenario</x:v>
       </x:c>
       <x:c r="B18" s="72" t="str">
         <x:v>%</x:v>
@@ -2701,13 +2701,13 @@
         <x:v>FORMULA</x:v>
       </x:c>
       <x:c r="E18" s="72" t="str">
-        <x:v>Half of current estimate: 2x relative error in the adverse direction.</x:v>
+        <x:v>Half of current commercial package-completion rate: 2x relative error in the adverse direction.</x:v>
       </x:c>
       <x:c r="F18" s="68"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="72" t="str">
-        <x:v>GM at containment error scenario</x:v>
+        <x:v>GM at package-completion error scenario</x:v>
       </x:c>
       <x:c r="B19" s="72" t="str">
         <x:v>%</x:v>
@@ -2720,7 +2720,7 @@
         <x:v>FORMULA</x:v>
       </x:c>
       <x:c r="E19" s="72" t="str">
-        <x:v>Shows whether a 2x error breaks the model.</x:v>
+        <x:v>Shows whether a 2x package-completion error breaks the model.</x:v>
       </x:c>
       <x:c r="F19" s="68"/>
     </x:row>
@@ -2732,13 +2732,13 @@
         <x:v>text</x:v>
       </x:c>
       <x:c r="C20" s="72" t="str">
-        <x:v>Completion proxy; 80% -&gt; 40% drops usage GM below 60%.</x:v>
+        <x:v>Package-completion scenario; 80% -&gt; 40% drops usage GM below 60%.</x:v>
       </x:c>
       <x:c r="D20" s="72" t="str">
         <x:v>RED TEAM</x:v>
       </x:c>
       <x:c r="E20" s="72" t="str">
-        <x:v>At 2x adverse error, completed jobs halve and fixed cost is spread over fewer jobs.</x:v>
+        <x:v>At 2x adverse package-completion error, completed commercial jobs halve and fixed cost is spread over fewer jobs.</x:v>
       </x:c>
       <x:c r="F20" s="68"/>
     </x:row>
@@ -2750,14 +2750,14 @@
         <x:v>check</x:v>
       </x:c>
       <x:c r="C21" s="78" t="str">
-        <x:f>IF(C19&gt;=C15,"PASS - withstands 2x adverse containment error","REMEDIATION - containment/price/cost action required")</x:f>
-        <x:v>REMEDIATION - containment/price/cost action required</x:v>
+        <x:f>IF(C19&gt;=C15,"PASS - withstands 2x adverse package-completion error","REMEDIATION - package-completion/price/cost action required")</x:f>
+        <x:v>REMEDIATION - package-completion/price/cost action required</x:v>
       </x:c>
       <x:c r="D21" s="72" t="str">
         <x:v>FORMULA</x:v>
       </x:c>
       <x:c r="E21" s="72" t="str">
-        <x:v>Proceed with paid pilot only while production completion evidence improves.</x:v>
+        <x:v>Proceed with paid pilot only while customer package-completion evidence improves.</x:v>
       </x:c>
       <x:c r="F21" s="68"/>
     </x:row>
@@ -2912,7 +2912,7 @@
         <x:v>FORMULA</x:v>
       </x:c>
       <x:c r="E30" s="72" t="str">
-        <x:v>Minutes displaced x labor rate x jobs attempted x containment.</x:v>
+        <x:v>Minutes displaced x labor rate x jobs attempted x commercial package-completion rate.</x:v>
       </x:c>
       <x:c r="F30" s="68"/>
     </x:row>
@@ -3043,33 +3043,33 @@
     </x:row>
     <x:row r="41" ht="22" customHeight="1">
       <x:c r="A41" s="70" t="str">
-        <x:v>Containment Sensitivity | variable usage price = 32,000 VND / completed job</x:v>
+        <x:v>Package-Completion Sensitivity | variable usage price = 32,000 VND / completed job</x:v>
       </x:c>
       <x:c r="B41" s="70" t="str">
-        <x:v>Containment Sensitivity | variable usage price = 32,000 VND / completed job</x:v>
+        <x:v>Package-Completion Sensitivity | variable usage price = 32,000 VND / completed job</x:v>
       </x:c>
       <x:c r="C41" s="70" t="str">
-        <x:v>Containment Sensitivity | variable usage price = 32,000 VND / completed job</x:v>
+        <x:v>Package-Completion Sensitivity | variable usage price = 32,000 VND / completed job</x:v>
       </x:c>
       <x:c r="D41" s="70" t="str">
-        <x:v>Containment Sensitivity | variable usage price = 32,000 VND / completed job</x:v>
+        <x:v>Package-Completion Sensitivity | variable usage price = 32,000 VND / completed job</x:v>
       </x:c>
       <x:c r="E41" s="70" t="str">
-        <x:v>Containment Sensitivity | variable usage price = 32,000 VND / completed job</x:v>
+        <x:v>Package-Completion Sensitivity | variable usage price = 32,000 VND / completed job</x:v>
       </x:c>
       <x:c r="F41" s="70" t="str">
-        <x:v>Containment Sensitivity | variable usage price = 32,000 VND / completed job</x:v>
+        <x:v>Package-Completion Sensitivity | variable usage price = 32,000 VND / completed job</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="73" t="str">
-        <x:v>Containment</x:v>
+        <x:v>Package completion rate</x:v>
       </x:c>
       <x:c r="B42" s="73" t="str">
-        <x:v>Completed jobs</x:v>
+        <x:v>Completed commercial jobs</x:v>
       </x:c>
       <x:c r="C42" s="73" t="str">
-        <x:v>Escalations</x:v>
+        <x:v>Modelled escalations</x:v>
       </x:c>
       <x:c r="D42" s="73" t="str">
         <x:v>Direct monthly cost</x:v>
@@ -3322,7 +3322,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R326d5a869c8147ed"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree69a64e7b514454"/>
 </x:worksheet>
 </file>
 
@@ -3557,10 +3557,10 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="72" t="str">
-        <x:v>Containment definition</x:v>
+        <x:v>Commercial billing job definition</x:v>
       </x:c>
       <x:c r="B15" s="72" t="str">
-        <x:v>Schema-valid grounded investigation package with required evidence/decision fields; customer final disposition recorded separately.</x:v>
+        <x:v>One completed grounded investigation package with required evidence/decision fields; customer final disposition recorded separately.</x:v>
       </x:c>
       <x:c r="C15" s="72" t="str">
         <x:v>P-015 metrics-pack core action and scope; adapted for the copilot billing boundary.</x:v>
@@ -3569,7 +3569,7 @@
         <x:v>DEFINITION</x:v>
       </x:c>
       <x:c r="E15" s="72" t="str">
-        <x:v>Bill only when objective package completion rule is met; do not treat human-gated review as autonomous completion.</x:v>
+        <x:v>Bill only when the objective package-completion rule is met; do not treat human-gated review as autonomous containment.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -4462,13 +4462,13 @@
         <x:v>46356</x:v>
       </x:c>
       <x:c r="D12" s="72" t="str">
-        <x:v>Containment</x:v>
+        <x:v>Package completion</x:v>
       </x:c>
       <x:c r="E12" s="72" t="str">
-        <x:v>&gt;=85% measured completion</x:v>
+        <x:v>&gt;=85% measured commercial package completion</x:v>
       </x:c>
       <x:c r="F12" s="72" t="str">
-        <x:v>Completion log with denominator</x:v>
+        <x:v>Completion log with denominator; autonomous containment and escalation reported separately</x:v>
       </x:c>
       <x:c r="G12" s="79" t="str">
         <x:v>PLANNED</x:v>

</xml_diff>